<commit_message>
Revised parameter inputs for template version of Jean et al. flouride model.
</commit_message>
<xml_diff>
--- a/Inputs/F_template_parameters_Model.xlsx
+++ b/Inputs/F_template_parameters_Model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/schlosser_paul_epa_gov/Documents/mcsim-5.6.5/PBPK_Model_Template_Mod/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="257" documentId="8_{7F8D94C6-EC2B-4A79-A22A-AD1B7807B962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BAEC706-8C59-4BC2-9C2F-BEF881BFFAC2}"/>
+  <xr:revisionPtr revIDLastSave="295" documentId="8_{7F8D94C6-EC2B-4A79-A22A-AD1B7807B962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0CD96151-D1AD-4DB3-9455-7E599C57FEA7}"/>
   <bookViews>
-    <workbookView xWindow="-23040" yWindow="45" windowWidth="25410" windowHeight="14640" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="24600" windowHeight="13290" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
   </bookViews>
   <sheets>
     <sheet name="Human4yo" sheetId="9" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="290">
   <si>
     <t>Code</t>
   </si>
@@ -874,9 +874,6 @@
     <t>Total plasma CL (L/h ~ kg/h; Jean 2016)</t>
   </si>
   <si>
-    <t>Tota urinary CL (L/h) V</t>
-  </si>
-  <si>
     <t>&lt;= Total bone CL (L/h)</t>
   </si>
   <si>
@@ -935,6 +932,12 @@
   </si>
   <si>
     <t>Below was copied, with limited translation, from the Jean et al. spreadsheet</t>
+  </si>
+  <si>
+    <t>used for kidney</t>
+  </si>
+  <si>
+    <t>Tota urinary [kidney] CL (L/h) from plasma; multiply by 1.333 to get CL from blood</t>
   </si>
 </sst>
 </file>
@@ -1091,7 +1094,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1127,6 +1130,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1263,10 +1267,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1709,7 +1709,7 @@
         <v>2</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1952,7 +1952,7 @@
         <v>103</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="J25" s="4"/>
     </row>
@@ -1981,7 +1981,7 @@
         <v>6926.2410142047056</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="J26" s="4"/>
     </row>
@@ -2045,6 +2045,9 @@
       <c r="D29">
         <v>0</v>
       </c>
+      <c r="E29">
+        <v>100</v>
+      </c>
       <c r="F29" s="4">
         <f>0.1 + 0.0222*age</f>
         <v>0.18880000000000002</v>
@@ -2091,6 +2094,14 @@
       <c r="D31">
         <v>0</v>
       </c>
+      <c r="F31" s="4">
+        <f>CLp*F$30</f>
+        <v>6.1336511205204829</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="H31" s="4"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
@@ -2109,7 +2120,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>52</v>
       </c>
@@ -2123,7 +2134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>53</v>
       </c>
@@ -2137,7 +2148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>54</v>
       </c>
@@ -2150,11 +2161,12 @@
       <c r="D35">
         <v>0</v>
       </c>
-      <c r="F35" s="4" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G35" s="4"/>
+      <c r="H35" s="4"/>
+      <c r="I35" s="4"/>
+      <c r="J35" s="4"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>165</v>
       </c>
@@ -2167,174 +2179,172 @@
       <c r="D36">
         <v>0</v>
       </c>
-      <c r="E36" s="4">
-        <f>F36/(BW^0.75)</f>
-        <v>0.17844448526169063</v>
-      </c>
-      <c r="F36" s="4">
+      <c r="G36" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B37" t="s">
+        <v>167</v>
+      </c>
+      <c r="C37" t="s">
+        <v>190</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="B38" t="s">
+        <v>57</v>
+      </c>
+      <c r="C38" t="s">
+        <v>46</v>
+      </c>
+      <c r="D38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="B39" t="s">
+        <v>58</v>
+      </c>
+      <c r="C39" t="s">
+        <v>59</v>
+      </c>
+      <c r="D39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="B40" t="s">
+        <v>60</v>
+      </c>
+      <c r="C40" t="s">
+        <v>36</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B41" t="s">
+        <v>61</v>
+      </c>
+      <c r="C41" t="s">
+        <v>189</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="F41" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B42" t="s">
+        <v>62</v>
+      </c>
+      <c r="C42" t="s">
+        <v>46</v>
+      </c>
+      <c r="D42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B43" t="s">
+        <v>63</v>
+      </c>
+      <c r="C43" t="s">
+        <v>244</v>
+      </c>
+      <c r="D43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B44" t="s">
+        <v>64</v>
+      </c>
+      <c r="C44" t="s">
+        <v>189</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+      <c r="F44" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="B45" t="s">
+        <v>65</v>
+      </c>
+      <c r="C45" t="s">
+        <v>46</v>
+      </c>
+      <c r="D45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A46" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="B46" t="s">
+        <v>204</v>
+      </c>
+      <c r="C46" t="s">
+        <v>244</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+      <c r="E46" s="4">
+        <f>F46*1.333/(E75*(BW^0.75))</f>
+        <v>46.606293058664804</v>
+      </c>
+      <c r="F46" s="4">
         <f>CLp*F29</f>
         <v>1.4275558820935248</v>
       </c>
-      <c r="G36" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B37" t="s">
-        <v>167</v>
-      </c>
-      <c r="C37" t="s">
-        <v>190</v>
-      </c>
-      <c r="D37">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="B38" t="s">
-        <v>57</v>
-      </c>
-      <c r="C38" t="s">
-        <v>46</v>
-      </c>
-      <c r="D38">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="B39" t="s">
-        <v>58</v>
-      </c>
-      <c r="C39" t="s">
-        <v>59</v>
-      </c>
-      <c r="D39">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="B40" t="s">
-        <v>60</v>
-      </c>
-      <c r="C40" t="s">
-        <v>36</v>
-      </c>
-      <c r="D40">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A41" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="B41" t="s">
-        <v>61</v>
-      </c>
-      <c r="C41" t="s">
-        <v>189</v>
-      </c>
-      <c r="D41">
-        <v>0</v>
-      </c>
-      <c r="F41" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A42" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="B42" t="s">
-        <v>62</v>
-      </c>
-      <c r="C42" t="s">
-        <v>46</v>
-      </c>
-      <c r="D42">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="B43" t="s">
-        <v>63</v>
-      </c>
-      <c r="C43" t="s">
-        <v>244</v>
-      </c>
-      <c r="D43">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="B44" t="s">
-        <v>64</v>
-      </c>
-      <c r="C44" t="s">
-        <v>189</v>
-      </c>
-      <c r="D44">
-        <v>0</v>
-      </c>
-      <c r="F44" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A45" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="B45" t="s">
-        <v>65</v>
-      </c>
-      <c r="C45" t="s">
-        <v>46</v>
-      </c>
-      <c r="D45">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="B46" t="s">
-        <v>204</v>
-      </c>
-      <c r="C46" t="s">
-        <v>244</v>
-      </c>
-      <c r="D46">
-        <v>0</v>
-      </c>
-      <c r="E46" s="4"/>
-      <c r="F46" s="4">
-        <f>CLp*F30</f>
-        <v>6.1336511205204829</v>
-      </c>
       <c r="G46" s="4" t="s">
-        <v>269</v>
+        <v>289</v>
       </c>
       <c r="H46" s="4"/>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I46" s="4"/>
+      <c r="J46" s="4"/>
+      <c r="K46" s="4"/>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>148</v>
       </c>
@@ -2351,7 +2361,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>149</v>
       </c>
@@ -2609,7 +2619,7 @@
         <v>216</v>
       </c>
       <c r="G66" s="4" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.25">
@@ -2649,16 +2659,8 @@
       <c r="D68">
         <v>1</v>
       </c>
-      <c r="E68" s="4">
-        <f>((4.214*BW^0.823)+(4.456*BW^0.795))/(BW*1000)</f>
-        <v>5.1037420752262702E-3</v>
-      </c>
       <c r="F68" t="s">
         <v>218</v>
-      </c>
-      <c r="G68" s="4">
-        <f>E68*BW</f>
-        <v>8.1659873203620323E-2</v>
       </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.25">
@@ -2692,7 +2694,7 @@
         <v>1</v>
       </c>
       <c r="E70" s="4">
-        <f>(((-0.005309*age+1.008*BW^0.493+BH^0.3765-7.952)+( 0.002331*age+0.1253*BW^0.8477+BH^0.3821-4.725))/(2*BW))-E67-E68</f>
+        <f>(((-0.005309*age+1.008*BW^0.493+BH^0.3765-7.952)+( 0.002331*age+0.1253*BW^0.8477+BH^0.3821-4.725))/(2*BW))-E67-E75</f>
         <v>9.9581643578766893E-2</v>
       </c>
       <c r="F70" t="s">
@@ -2767,11 +2769,18 @@
       <c r="D74">
         <v>1</v>
       </c>
-      <c r="F74" t="s">
-        <v>223</v>
+      <c r="E74" s="4">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="F74" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="G74" s="4">
+        <f>E74*BW</f>
+        <v>1.1200000000000001</v>
       </c>
       <c r="J74" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="75" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2788,18 +2797,19 @@
         <v>1</v>
       </c>
       <c r="E75" s="4">
-        <v>7.0000000000000007E-2</v>
+        <f>((4.214*BW^0.823)+(4.456*BW^0.795))/(BW*1000)</f>
+        <v>5.1037420752262702E-3</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>260</v>
+        <v>288</v>
       </c>
       <c r="G75" s="4">
         <f>E75*BW</f>
-        <v>1.1200000000000001</v>
+        <v>8.1659873203620323E-2</v>
       </c>
       <c r="J75" s="9"/>
       <c r="K75" s="10" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="L75" s="11"/>
     </row>
@@ -2821,7 +2831,7 @@
         <v>0.79931461434600681</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="G76" s="7">
         <f>E76*BW</f>
@@ -2829,10 +2839,10 @@
       </c>
       <c r="J76" s="12"/>
       <c r="K76" s="13" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="L76" s="14" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.25">
@@ -2856,10 +2866,10 @@
         <v>116.71859368947428</v>
       </c>
       <c r="H77" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="J77" s="15" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="K77" s="13">
         <f>0.00119*BW-0.0004302</f>
@@ -2895,7 +2905,7 @@
         <v>0.38272</v>
       </c>
       <c r="J78" s="15" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="K78" s="13">
         <f>0.0000001017*((BH^0.6862*BW^0.3561*242.7+BH^0.664*BW^0.3851*242.7)/2)^1.42</f>
@@ -2919,18 +2929,11 @@
       <c r="D79">
         <v>0</v>
       </c>
-      <c r="E79" s="4">
-        <v>0.18</v>
-      </c>
       <c r="F79" t="s">
         <v>218</v>
       </c>
-      <c r="G79" s="7">
-        <f>E79*Qct</f>
-        <v>21.009346864105368</v>
-      </c>
       <c r="J79" s="15" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K79" s="13">
         <f>((6.78*(surface/10000)^1.629-0.001492*age+3.58)+(0.2598*BW+0.1206*BH-0.0043*age-11.1)/1.04)/2</f>
@@ -2955,7 +2958,7 @@
         <v>0</v>
       </c>
       <c r="E80" s="5">
-        <f>1-SUM(E78:E79,E85:E86)</f>
+        <f>1-SUM(E78,E84:E86)</f>
         <v>0.76216599738664981</v>
       </c>
       <c r="F80" t="s">
@@ -2969,7 +2972,7 @@
         <v>256</v>
       </c>
       <c r="J80" s="15" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="K80" s="13">
         <f>SUM(K77:K79)</f>
@@ -3023,10 +3026,10 @@
         <v>221</v>
       </c>
       <c r="K82" s="17" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="L82" s="4" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="M82" s="4"/>
       <c r="N82" s="4"/>
@@ -3048,10 +3051,10 @@
         <v>222</v>
       </c>
       <c r="K83" s="17" t="s">
+        <v>283</v>
+      </c>
+      <c r="L83" s="4" t="s">
         <v>284</v>
-      </c>
-      <c r="L83" s="4" t="s">
-        <v>285</v>
       </c>
       <c r="M83" s="4"/>
       <c r="N83" s="4"/>
@@ -3069,9 +3072,22 @@
       <c r="D84">
         <v>0</v>
       </c>
-      <c r="F84" t="s">
-        <v>223</v>
-      </c>
+      <c r="E84" s="6">
+        <v>0.05</v>
+      </c>
+      <c r="F84" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="G84" s="7">
+        <f>E84*Qct</f>
+        <v>5.8359296844737143</v>
+      </c>
+      <c r="H84" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="I84" s="6"/>
+      <c r="J84" s="6"/>
+      <c r="K84" s="6"/>
     </row>
     <row r="85" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
@@ -3086,15 +3102,15 @@
       <c r="D85">
         <v>0</v>
       </c>
-      <c r="E85" s="6">
-        <v>0.05</v>
+      <c r="E85" s="4">
+        <v>0.18</v>
       </c>
       <c r="F85" s="4" t="s">
-        <v>260</v>
+        <v>288</v>
       </c>
       <c r="G85" s="7">
         <f>E85*Qct</f>
-        <v>5.8359296844737143</v>
+        <v>21.009346864105368</v>
       </c>
       <c r="H85" s="6" t="s">
         <v>261</v>
@@ -3121,7 +3137,7 @@
         <v>4.5550049155351395E-3</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="G86" s="7">
         <f>L81</f>
@@ -3156,7 +3172,7 @@
         <v>216</v>
       </c>
       <c r="G88" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="H88" s="4"/>
     </row>
@@ -3191,15 +3207,9 @@
       <c r="D90">
         <v>1</v>
       </c>
-      <c r="E90" s="7">
-        <f t="shared" ref="E90:E91" si="0">G90*1.333</f>
-        <v>5.54528</v>
-      </c>
+      <c r="E90" s="19"/>
       <c r="F90" t="s">
         <v>218</v>
-      </c>
-      <c r="G90">
-        <v>4.16</v>
       </c>
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.25">
@@ -3213,7 +3223,7 @@
         <v>1</v>
       </c>
       <c r="E91" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E90:E91" si="0">G91*1.333</f>
         <v>1.10639</v>
       </c>
       <c r="F91" t="s">
@@ -3278,9 +3288,15 @@
       <c r="D95">
         <v>1</v>
       </c>
-      <c r="E95" s="18"/>
-      <c r="F95" t="s">
-        <v>223</v>
+      <c r="E95" s="7">
+        <f t="shared" ref="E95:E96" si="1">G95*1.333</f>
+        <v>1333</v>
+      </c>
+      <c r="F95" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="G95">
+        <v>1000</v>
       </c>
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.25">
@@ -3294,14 +3310,14 @@
         <v>1</v>
       </c>
       <c r="E96" s="7">
-        <f t="shared" ref="E96:E97" si="1">G96*1.333</f>
-        <v>1333</v>
+        <f t="shared" si="1"/>
+        <v>5.54528</v>
       </c>
       <c r="F96" s="4" t="s">
-        <v>260</v>
+        <v>288</v>
       </c>
       <c r="G96">
-        <v>1000</v>
+        <v>4.16</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
@@ -3315,11 +3331,11 @@
         <v>1</v>
       </c>
       <c r="E97" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="E96:E97" si="2">G97*1.333</f>
         <v>0.83979000000000004</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="G97">
         <v>0.63</v>
@@ -5083,20 +5099,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5efa0b4590ceb4068c523eef838cbf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d32b47d5805bf9e4ccfb00021215c68" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -5569,6 +5571,20 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -5615,22 +5631,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90A172F1-773B-43BF-8B86-8CD1537A96AE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5653,6 +5653,22 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Added to explanatory comments in Flouride model input spreadsheet.
</commit_message>
<xml_diff>
--- a/Inputs/F_template_parameters_Model.xlsx
+++ b/Inputs/F_template_parameters_Model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/schlosser_paul_epa_gov/Documents/mcsim-5.6.5/PBPK_Model_Template_Mod/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="295" documentId="8_{7F8D94C6-EC2B-4A79-A22A-AD1B7807B962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0CD96151-D1AD-4DB3-9455-7E599C57FEA7}"/>
+  <xr:revisionPtr revIDLastSave="311" documentId="8_{7F8D94C6-EC2B-4A79-A22A-AD1B7807B962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF2E9500-7459-405E-94AF-6D9AA4ACA781}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="24600" windowHeight="13290" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
+    <workbookView xWindow="3420" yWindow="1830" windowWidth="24600" windowHeight="13290" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
   </bookViews>
   <sheets>
     <sheet name="Human4yo" sheetId="9" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="291">
   <si>
     <t>Code</t>
   </si>
@@ -922,15 +922,9 @@
     <t>volume above</t>
   </si>
   <si>
-    <t>x Vtf/"Total" volume</t>
-  </si>
-  <si>
     <t>^ "Total" blood flow above</t>
   </si>
   <si>
-    <t>Tissue:plasma coeffs</t>
-  </si>
-  <si>
     <t>Below was copied, with limited translation, from the Jean et al. spreadsheet</t>
   </si>
   <si>
@@ -938,6 +932,15 @@
   </si>
   <si>
     <t>Tota urinary [kidney] CL (L/h) from plasma; multiply by 1.333 to get CL from blood</t>
+  </si>
+  <si>
+    <t>k_met_omc (E46) is also divided by V_omc (E75) and by BW^0.75 to convert CL to a rate 1st order scaled rate constant; it is multiplied by V_omc x BW / BW^0.25 in the code.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      x Vtf/"Total" volume</t>
+  </si>
+  <si>
+    <t>Tissue:plasma coeffs; multiplied by 1.3333 to get tissue:blood PCs</t>
   </si>
 </sst>
 </file>
@@ -947,7 +950,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -955,8 +958,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -984,6 +995,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1094,7 +1111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1130,7 +1147,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1267,6 +1293,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1566,7 +1596,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ADCAA70-43B6-4F02-AE2A-67A6EACE5958}">
-  <dimension ref="A1:N105"/>
+  <dimension ref="A1:O105"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -2120,7 +2150,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>52</v>
       </c>
@@ -2134,7 +2164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>53</v>
       </c>
@@ -2148,7 +2178,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>54</v>
       </c>
@@ -2166,7 +2196,7 @@
       <c r="I35" s="4"/>
       <c r="J35" s="4"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>165</v>
       </c>
@@ -2183,7 +2213,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>56</v>
       </c>
@@ -2197,7 +2227,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>237</v>
       </c>
@@ -2211,7 +2241,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>236</v>
       </c>
@@ -2225,7 +2255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>238</v>
       </c>
@@ -2239,7 +2269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>143</v>
       </c>
@@ -2256,7 +2286,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>144</v>
       </c>
@@ -2270,7 +2300,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>145</v>
       </c>
@@ -2284,7 +2314,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>146</v>
       </c>
@@ -2301,7 +2331,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>147</v>
       </c>
@@ -2314,8 +2344,18 @@
       <c r="D45">
         <v>1</v>
       </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="F45" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="G45" s="4"/>
+      <c r="H45" s="4"/>
+      <c r="I45" s="4"/>
+      <c r="J45" s="4"/>
+      <c r="K45" s="4"/>
+      <c r="L45" s="4"/>
+      <c r="M45" s="4"/>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>203</v>
       </c>
@@ -2337,14 +2377,15 @@
         <v>1.4275558820935248</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="H46" s="4"/>
       <c r="I46" s="4"/>
       <c r="J46" s="4"/>
       <c r="K46" s="4"/>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L46" s="4"/>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>148</v>
       </c>
@@ -2361,7 +2402,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>149</v>
       </c>
@@ -2585,7 +2626,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>82</v>
       </c>
@@ -2602,7 +2643,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>89</v>
       </c>
@@ -2622,7 +2663,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>90</v>
       </c>
@@ -2646,7 +2687,7 @@
         <v>0.41599999999999998</v>
       </c>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>91</v>
       </c>
@@ -2663,7 +2704,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>92</v>
       </c>
@@ -2680,7 +2721,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>93</v>
       </c>
@@ -2705,7 +2746,7 @@
         <v>1.5933062972602703</v>
       </c>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>94</v>
       </c>
@@ -2722,7 +2763,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>95</v>
       </c>
@@ -2739,7 +2780,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>96</v>
       </c>
@@ -2756,7 +2797,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="74" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>97</v>
       </c>
@@ -2779,11 +2820,16 @@
         <f>E74*BW</f>
         <v>1.1200000000000001</v>
       </c>
-      <c r="J74" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="75" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J74" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="K74" s="4"/>
+      <c r="L74" s="4"/>
+      <c r="M74" s="4"/>
+      <c r="N74" s="4"/>
+      <c r="O74" s="4"/>
+    </row>
+    <row r="75" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>98</v>
       </c>
@@ -2801,7 +2847,7 @@
         <v>5.1037420752262702E-3</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="G75" s="4">
         <f>E75*BW</f>
@@ -2813,7 +2859,7 @@
       </c>
       <c r="L75" s="11"/>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>151</v>
       </c>
@@ -2845,7 +2891,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>104</v>
       </c>
@@ -2880,7 +2926,7 @@
         <v>5.5829400000000009E-4</v>
       </c>
     </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>105</v>
       </c>
@@ -2916,7 +2962,7 @@
         <v>7.6608431731805898E-2</v>
       </c>
     </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>106</v>
       </c>
@@ -2944,7 +2990,7 @@
         <v>0.18829093630147836</v>
       </c>
     </row>
-    <row r="80" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>107</v>
       </c>
@@ -2971,14 +3017,14 @@
       <c r="H80" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="J80" s="15" t="s">
+      <c r="J80" s="19" t="s">
         <v>279</v>
       </c>
-      <c r="K80" s="13">
+      <c r="K80" s="20">
         <f>SUM(K77:K79)</f>
         <v>6.3856352093374129</v>
       </c>
-      <c r="L80" s="14">
+      <c r="L80" s="21">
         <f>SUM(L77:L79)</f>
         <v>0.26545766203328425</v>
       </c>
@@ -3029,7 +3075,7 @@
         <v>282</v>
       </c>
       <c r="L82" s="4" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="M82" s="4"/>
       <c r="N82" s="4"/>
@@ -3054,7 +3100,7 @@
         <v>283</v>
       </c>
       <c r="L83" s="4" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="M83" s="4"/>
       <c r="N83" s="4"/>
@@ -3106,18 +3152,12 @@
         <v>0.18</v>
       </c>
       <c r="F85" s="4" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="G85" s="7">
         <f>E85*Qct</f>
         <v>21.009346864105368</v>
       </c>
-      <c r="H85" s="6" t="s">
-        <v>261</v>
-      </c>
-      <c r="I85" s="6"/>
-      <c r="J85" s="6"/>
-      <c r="K85" s="6"/>
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
@@ -3171,10 +3211,13 @@
       <c r="F88" t="s">
         <v>216</v>
       </c>
-      <c r="G88" s="4" t="s">
-        <v>286</v>
-      </c>
-      <c r="H88" s="4"/>
+      <c r="G88" s="22" t="s">
+        <v>290</v>
+      </c>
+      <c r="H88" s="22"/>
+      <c r="I88" s="22"/>
+      <c r="J88" s="22"/>
+      <c r="K88" s="22"/>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
@@ -3193,7 +3236,7 @@
       <c r="F89" t="s">
         <v>217</v>
       </c>
-      <c r="G89">
+      <c r="G89" s="22">
         <v>0.98</v>
       </c>
     </row>
@@ -3207,10 +3250,11 @@
       <c r="D90">
         <v>1</v>
       </c>
-      <c r="E90" s="19"/>
+      <c r="E90" s="18"/>
       <c r="F90" t="s">
         <v>218</v>
       </c>
+      <c r="G90" s="22"/>
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
@@ -3223,13 +3267,13 @@
         <v>1</v>
       </c>
       <c r="E91" s="7">
-        <f t="shared" ref="E90:E91" si="0">G91*1.333</f>
+        <f t="shared" ref="E91" si="0">G91*1.333</f>
         <v>1.10639</v>
       </c>
       <c r="F91" t="s">
         <v>259</v>
       </c>
-      <c r="G91">
+      <c r="G91" s="22">
         <v>0.83</v>
       </c>
     </row>
@@ -3247,6 +3291,7 @@
       <c r="F92" t="s">
         <v>220</v>
       </c>
+      <c r="G92" s="22"/>
     </row>
     <row r="93" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
@@ -3262,6 +3307,7 @@
       <c r="F93" t="s">
         <v>221</v>
       </c>
+      <c r="G93" s="22"/>
     </row>
     <row r="94" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
@@ -3277,6 +3323,7 @@
       <c r="F94" t="s">
         <v>222</v>
       </c>
+      <c r="G94" s="22"/>
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
@@ -3295,7 +3342,7 @@
       <c r="F95" s="4" t="s">
         <v>260</v>
       </c>
-      <c r="G95">
+      <c r="G95" s="22">
         <v>1000</v>
       </c>
     </row>
@@ -3314,9 +3361,9 @@
         <v>5.54528</v>
       </c>
       <c r="F96" s="4" t="s">
-        <v>288</v>
-      </c>
-      <c r="G96">
+        <v>286</v>
+      </c>
+      <c r="G96" s="22">
         <v>4.16</v>
       </c>
     </row>
@@ -3331,13 +3378,13 @@
         <v>1</v>
       </c>
       <c r="E97" s="7">
-        <f t="shared" ref="E96:E97" si="2">G97*1.333</f>
+        <f t="shared" ref="E97" si="2">G97*1.333</f>
         <v>0.83979000000000004</v>
       </c>
       <c r="F97" s="4" t="s">
         <v>271</v>
       </c>
-      <c r="G97">
+      <c r="G97" s="22">
         <v>0.63</v>
       </c>
     </row>
@@ -5099,6 +5146,65 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
+    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </j747ac98061d40f0aa7bd47e1db5675d>
+    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
+    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
+    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
+    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creator>
+    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </EPA_x0020_Contributor>
+    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </e3f09c3df709400db2417a7161762d62>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5efa0b4590ceb4068c523eef838cbf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d32b47d5805bf9e4ccfb00021215c68" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -5571,66 +5677,38 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
-    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </j747ac98061d40f0aa7bd47e1db5675d>
-    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
-    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
-    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
-    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creator>
-    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </EPA_x0020_Contributor>
-    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </e3f09c3df709400db2417a7161762d62>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90A172F1-773B-43BF-8B86-8CD1537A96AE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5651,35 +5729,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
-    <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
-    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Some equations simplified (algebra) in the the flouride parameter input spreadsheet.
</commit_message>
<xml_diff>
--- a/Inputs/F_template_parameters_Model.xlsx
+++ b/Inputs/F_template_parameters_Model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/schlosser_paul_epa_gov/Documents/mcsim-5.6.5/PBPK_Model_Template_Mod/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="311" documentId="8_{7F8D94C6-EC2B-4A79-A22A-AD1B7807B962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF2E9500-7459-405E-94AF-6D9AA4ACA781}"/>
+  <xr:revisionPtr revIDLastSave="313" documentId="8_{7F8D94C6-EC2B-4A79-A22A-AD1B7807B962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF183F8B-7B2C-4498-A91A-80194D400391}"/>
   <bookViews>
-    <workbookView xWindow="3420" yWindow="1830" windowWidth="24600" windowHeight="13290" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
+    <workbookView xWindow="1725" yWindow="225" windowWidth="24600" windowHeight="13290" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
   </bookViews>
   <sheets>
     <sheet name="Human4yo" sheetId="9" r:id="rId1"/>
@@ -5146,65 +5146,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
-    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </j747ac98061d40f0aa7bd47e1db5675d>
-    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
-    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
-    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
-    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creator>
-    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </EPA_x0020_Contributor>
-    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </e3f09c3df709400db2417a7161762d62>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5efa0b4590ceb4068c523eef838cbf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d32b47d5805bf9e4ccfb00021215c68" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -5677,38 +5618,66 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
-    <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
-    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
+    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </j747ac98061d40f0aa7bd47e1db5675d>
+    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
+    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
+    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
+    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creator>
+    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </EPA_x0020_Contributor>
+    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </e3f09c3df709400db2417a7161762d62>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90A172F1-773B-43BF-8B86-8CD1537A96AE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5729,4 +5698,35 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Revised comments and calculations in Flouride_template... parameter spreadsheet.
</commit_message>
<xml_diff>
--- a/Inputs/F_template_parameters_Model.xlsx
+++ b/Inputs/F_template_parameters_Model.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="313" documentId="8_{7F8D94C6-EC2B-4A79-A22A-AD1B7807B962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF183F8B-7B2C-4498-A91A-80194D400391}"/>
   <bookViews>
-    <workbookView xWindow="1725" yWindow="225" windowWidth="24600" windowHeight="13290" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
+    <workbookView xWindow="1080" yWindow="293" windowWidth="24600" windowHeight="13294" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
   </bookViews>
   <sheets>
     <sheet name="Human4yo" sheetId="9" r:id="rId1"/>
@@ -5146,6 +5146,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5efa0b4590ceb4068c523eef838cbf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d32b47d5805bf9e4ccfb00021215c68" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -5618,21 +5623,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
@@ -5677,7 +5668,24 @@
 </p:properties>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90A172F1-773B-43BF-8B86-8CD1537A96AE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5700,23 +5708,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -5729,4 +5721,12 @@
     <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>